<commit_message>
Adding 2024 male data
</commit_message>
<xml_diff>
--- a/RawData/MaleMonthlyAssaults.xlsx
+++ b/RawData/MaleMonthlyAssaults.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Desktop/TexasMortality/RawData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ainsl/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C00918E6-F310-EF48-B7E9-074FEBCA4D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97490B66-F61A-C243-A2AE-764A0E1F2B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" xr2:uid="{FDCCCDDD-5AF2-1241-93B7-8C4D33297932}"/>
+    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{A0421283-1E6D-3B42-BC06-37B4F65416C1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Provisional Mortality Statistic" sheetId="1" r:id="rId1"/>
-    <sheet name="Data Details" sheetId="2" r:id="rId2"/>
+    <sheet name="MaleMonthlyAssaults" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="224">
   <si>
     <t>Notes</t>
   </si>
@@ -41,6 +40,12 @@
     <t>Crude Rate</t>
   </si>
   <si>
+    <t>Crude Rate Lower 95% Confidence Interval</t>
+  </si>
+  <si>
+    <t>Crude Rate Upper 95% Confidence Interval</t>
+  </si>
+  <si>
     <t>Jan., 2018</t>
   </si>
   <si>
@@ -476,13 +481,82 @@
     <t>2023/12</t>
   </si>
   <si>
-    <t>Total</t>
+    <t xml:space="preserve">Jan., 2024 </t>
+  </si>
+  <si>
+    <t>2024/01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feb., 2024 </t>
+  </si>
+  <si>
+    <t>2024/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mar., 2024 </t>
+  </si>
+  <si>
+    <t>2024/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apr., 2024 </t>
+  </si>
+  <si>
+    <t>2024/04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May, 2024 </t>
+  </si>
+  <si>
+    <t>2024/05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun., 2024 </t>
+  </si>
+  <si>
+    <t>2024/06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul., 2024 </t>
+  </si>
+  <si>
+    <t>2024/07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug., 2024 </t>
+  </si>
+  <si>
+    <t>2024/08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep., 2024 </t>
+  </si>
+  <si>
+    <t>2024/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct., 2024 </t>
+  </si>
+  <si>
+    <t>2024/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov., 2024 </t>
+  </si>
+  <si>
+    <t>2024/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dec., 2024 </t>
+  </si>
+  <si>
+    <t>2024/12</t>
   </si>
   <si>
     <t>---</t>
   </si>
   <si>
-    <t>Dataset: Provisional Mortality Statistics, 2018 through Last Week</t>
+    <t>Dataset: Multiple Cause of Death, 2018-2024, Single Race</t>
   </si>
   <si>
     <t>Query Parameters:</t>
@@ -491,28 +565,25 @@
     <t>MCD - ICD-10 Codes: X85-Y09 (Assault)</t>
   </si>
   <si>
-    <t>Residence States: Texas (48)</t>
-  </si>
-  <si>
     <t>Sex: Male</t>
   </si>
   <si>
+    <t>States: Texas (48)</t>
+  </si>
+  <si>
     <t>Ten-Year Age Groups: 15-24 years; 25-34 years; 35-44 years</t>
   </si>
   <si>
-    <t>Year/Month: 2018; 2019; 2020; 2021; 2022; 2023</t>
-  </si>
-  <si>
     <t>Group By: Month</t>
   </si>
   <si>
-    <t>Show Totals: True</t>
-  </si>
-  <si>
-    <t>Show Zero Values: False</t>
-  </si>
-  <si>
-    <t>Show Suppressed: False</t>
+    <t>Show Totals: False</t>
+  </si>
+  <si>
+    <t>Show Zero Values: True</t>
+  </si>
+  <si>
+    <t>Show Suppressed: True</t>
   </si>
   <si>
     <t>Calculate Rates Per: 100,000</t>
@@ -521,34 +592,34 @@
     <t>Rate Options: Default intercensal populations for years 2001-2009 (except Infant Age Groups)</t>
   </si>
   <si>
-    <t>Help: See http://wonder.cdc.gov/wonder/help/mcd-provisional.html for more information.</t>
-  </si>
-  <si>
-    <t>Query Date: Feb 1, 2026 11:22:25 PM</t>
+    <t>Help: See http://wonder.cdc.gov/wonder/help/mcd-expanded.html for more information.</t>
+  </si>
+  <si>
+    <t>Query Date: May 10, 2026 3:22:49 PM</t>
   </si>
   <si>
     <t>Suggested Citation: Centers for Disease Control and Prevention, National Center for Health Statistics. National Vital Statistics</t>
   </si>
   <si>
-    <t>System, Provisional Mortality on CDC WONDER Online Database. Data are from the final Multiple Cause of Death Files, 2018-2023,</t>
-  </si>
-  <si>
-    <t>and from provisional data for years 2024 and later, as compiled from data provided by the 57 vital statistics jurisdictions</t>
-  </si>
-  <si>
-    <t>through the Vital Statistics Cooperative Program. Accessed at http://wonder.cdc.gov/mcd-icd10-provisional.html on Feb 1, 2026</t>
+    <t>System, Mortality 2018-2024 on CDC WONDER Online Database, released in 2026. Data are from the Multiple Cause of Death Files,</t>
+  </si>
+  <si>
+    <t>2018-2024, as compiled from data provided by the 57 vital statistics jurisdictions through the Vital Statistics Cooperative</t>
+  </si>
+  <si>
+    <t>Program. Accessed at http://wonder.cdc.gov/mcd-icd10-expanded.html on May 10, 2026 3:22:49 PM</t>
   </si>
   <si>
     <t>Caveats:</t>
   </si>
   <si>
-    <t>1. Population and rates are labeled 'Not Applicable' when location of Death's Occurrence, Autopsy, Place of Death, Weekday or</t>
-  </si>
-  <si>
-    <t>Month are grouped by or limited, due to lack of a valid population. More information:</t>
-  </si>
-  <si>
-    <t>http://wonder.cdc.gov/wonder/help/mcd-provisional.html#NotApplicableRates.</t>
+    <t>1. Population and rates are labeled 'Not Applicable' when Autopsy, Place of Death, Education, Industry, Usual Occupation,</t>
+  </si>
+  <si>
+    <t>Weekday or Month are grouped by or limited, due to lack of a valid population. More information:</t>
+  </si>
+  <si>
+    <t>http://wonder.cdc.gov/wonder/help/mcd-expanded.html#NotApplicableRates.</t>
   </si>
   <si>
     <t>2. Deaths of persons with Age "Not Stated" are included in "All" counts and rates, but are not distributed among age groups,</t>
@@ -557,10 +628,16 @@
     <t>so are not included in age-specific counts, age-specific rates or in any age-adjusted rates. More information:</t>
   </si>
   <si>
-    <t>http://wonder.cdc.gov/wonder/help/mcd-provisional.html#Not Stated.</t>
-  </si>
-  <si>
-    <t>3. On March 11, 2021, the 2019 mortality data on CDC WONDER was updated with the 2019 mortality data updated by NCHS on March 4,</t>
+    <t>http://wonder.cdc.gov/wonder/help/mcd-expanded.html#Not Stated.</t>
+  </si>
+  <si>
+    <t>3. The method used to calculate 95% confidence intervals is documented here: More information:</t>
+  </si>
+  <si>
+    <t>http://wonder.cdc.gov/wonder/help/mcd-expanded.html#Confidence-Intervals.</t>
+  </si>
+  <si>
+    <t>4. On March 11, 2021, the 2019 mortality data on CDC WONDER was updated with the 2019 mortality data updated by NCHS on March 4,</t>
   </si>
   <si>
     <t>2021 to include corrected information for residents of Texas affecting 5 records previously coded to cause code *U01.4,</t>
@@ -575,7 +652,31 @@
     <t>unspecified firearm discharge, ICD-10 code X95. The corrected final death records replaces the data released on December 22,</t>
   </si>
   <si>
-    <t>4. After the creation of the final 2023 dataset, North Carolina updated the cause of death information for over 900 death</t>
+    <t>5. The U.S. - Mexico Border Regions distinguish between counties near the U.S. - Mexico border in the border states of Arizona,</t>
+  </si>
+  <si>
+    <t>California, New Mexico, and Texas, and other areas. To simplify the Border region analysis, two mutually exclusive regions</t>
+  </si>
+  <si>
+    <t>within the United States are available: 1) U.S. - Mexico Border Region (i.e., 44 counties within 100 kilometers (62 miles) of</t>
+  </si>
+  <si>
+    <t>the U.S. - Mexico border), and 2) the U.S. Non-Border Region with the remaining counties of the selected four border states. The</t>
+  </si>
+  <si>
+    <t>Border counties selection was based on the 1983 La Paz Agreement:</t>
+  </si>
+  <si>
+    <t>https://www.epa.gov/sites/production/files/2015-09/documents/lapazagreement.pdf.. (i.e., counties for each state which fall</t>
+  </si>
+  <si>
+    <t>within 100 kilometers of the Border). Statistics are also available by each of the USA border counties along the U.S.-Mexico</t>
+  </si>
+  <si>
+    <t>area.</t>
+  </si>
+  <si>
+    <t>6. After the creation of the final 2023 dataset, North Carolina updated the cause of death information for over 900 death</t>
   </si>
   <si>
     <t>certificates to include a cause of death code indicating drug overdose (ICD-10 underlying cause-of-death codes: X40-X44,</t>
@@ -591,16 +692,13 @@
   </si>
   <si>
     <t>100,000 population. These deaths will not be updated on the final mortality datasets.</t>
-  </si>
-  <si>
-    <t>5. Deaths occurring through January 17, 2026 as of January 25, 2026.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -731,13 +829,6 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1084,11 +1175,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="19" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="19" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1463,11 +1551,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8ECFF3A-9FE1-484A-BE5D-65634DCBF80C}">
-  <dimension ref="A1:F98"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15EAE24-6CE1-1C4D-9646-49F414A56709}">
+  <dimension ref="A1:H137"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1486,1757 +1574,2206 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2">
         <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4">
         <v>90</v>
       </c>
       <c r="E4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5">
         <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D6">
         <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D7">
         <v>82</v>
       </c>
       <c r="E7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D8">
         <v>78</v>
       </c>
       <c r="E8" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9">
         <v>71</v>
       </c>
       <c r="E9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D10">
         <v>70</v>
       </c>
       <c r="E10" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D11">
         <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D12">
         <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13">
         <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D14">
         <v>73</v>
       </c>
       <c r="E14" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D15">
         <v>74</v>
       </c>
       <c r="E15" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D16">
         <v>82</v>
       </c>
       <c r="E16" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G16" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D17">
         <v>65</v>
       </c>
       <c r="E17" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D18">
         <v>98</v>
       </c>
       <c r="E18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G18" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D19">
         <v>80</v>
       </c>
       <c r="E19" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D20">
         <v>67</v>
       </c>
       <c r="E20" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D21">
         <v>77</v>
       </c>
       <c r="E21" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G21" t="s">
+        <v>10</v>
+      </c>
+      <c r="H21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C22" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D22">
         <v>89</v>
       </c>
       <c r="E22" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F22" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G22" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D23">
         <v>81</v>
       </c>
       <c r="E23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G23" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C24" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D24">
         <v>95</v>
       </c>
       <c r="E24" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G24" t="s">
+        <v>10</v>
+      </c>
+      <c r="H24" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D25">
         <v>103</v>
       </c>
       <c r="E25" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C26" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D26">
         <v>104</v>
       </c>
       <c r="E26" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G26" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D27">
         <v>75</v>
       </c>
       <c r="E27" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G27" t="s">
+        <v>10</v>
+      </c>
+      <c r="H27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D28">
         <v>94</v>
       </c>
       <c r="E28" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G28" t="s">
+        <v>10</v>
+      </c>
+      <c r="H28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D29">
         <v>95</v>
       </c>
       <c r="E29" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C30" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D30">
         <v>107</v>
       </c>
       <c r="E30" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H30" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C31" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D31">
         <v>102</v>
       </c>
       <c r="E31" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F31" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G31" t="s">
+        <v>10</v>
+      </c>
+      <c r="H31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D32">
         <v>108</v>
       </c>
       <c r="E32" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F32" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G32" t="s">
+        <v>10</v>
+      </c>
+      <c r="H32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D33">
         <v>113</v>
       </c>
       <c r="E33" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F33" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G33" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C34" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D34">
         <v>100</v>
       </c>
       <c r="E34" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G34" t="s">
+        <v>10</v>
+      </c>
+      <c r="H34" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D35">
         <v>135</v>
       </c>
       <c r="E35" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F35" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G35" t="s">
+        <v>10</v>
+      </c>
+      <c r="H35" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C36" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D36">
         <v>136</v>
       </c>
       <c r="E36" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G36" t="s">
+        <v>10</v>
+      </c>
+      <c r="H36" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C37" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D37">
         <v>137</v>
       </c>
       <c r="E37" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F37" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G37" t="s">
+        <v>10</v>
+      </c>
+      <c r="H37" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D38">
         <v>127</v>
       </c>
       <c r="E38" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F38" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G38" t="s">
+        <v>10</v>
+      </c>
+      <c r="H38" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C39" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D39">
         <v>99</v>
       </c>
       <c r="E39" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F39" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G39" t="s">
+        <v>10</v>
+      </c>
+      <c r="H39" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D40">
         <v>104</v>
       </c>
       <c r="E40" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G40" t="s">
+        <v>10</v>
+      </c>
+      <c r="H40" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D41">
         <v>124</v>
       </c>
       <c r="E41" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F41" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G41" t="s">
+        <v>10</v>
+      </c>
+      <c r="H41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C42" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D42">
         <v>137</v>
       </c>
       <c r="E42" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G42" t="s">
+        <v>10</v>
+      </c>
+      <c r="H42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D43">
         <v>131</v>
       </c>
       <c r="E43" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G43" t="s">
+        <v>10</v>
+      </c>
+      <c r="H43" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C44" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D44">
         <v>119</v>
       </c>
       <c r="E44" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F44" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G44" t="s">
+        <v>10</v>
+      </c>
+      <c r="H44" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D45">
         <v>119</v>
       </c>
       <c r="E45" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G45" t="s">
+        <v>10</v>
+      </c>
+      <c r="H45" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D46">
         <v>136</v>
       </c>
       <c r="E46" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F46" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G46" t="s">
+        <v>10</v>
+      </c>
+      <c r="H46" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C47" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D47">
         <v>135</v>
       </c>
       <c r="E47" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F47" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G47" t="s">
+        <v>10</v>
+      </c>
+      <c r="H47" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C48" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D48">
         <v>115</v>
       </c>
       <c r="E48" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F48" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G48" t="s">
+        <v>10</v>
+      </c>
+      <c r="H48" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C49" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D49">
         <v>136</v>
       </c>
       <c r="E49" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F49" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G49" t="s">
+        <v>10</v>
+      </c>
+      <c r="H49" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C50" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D50">
         <v>134</v>
       </c>
       <c r="E50" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F50" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G50" t="s">
+        <v>10</v>
+      </c>
+      <c r="H50" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C51" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D51">
         <v>109</v>
       </c>
       <c r="E51" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F51" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G51" t="s">
+        <v>10</v>
+      </c>
+      <c r="H51" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C52" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D52">
         <v>99</v>
       </c>
       <c r="E52" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G52" t="s">
+        <v>10</v>
+      </c>
+      <c r="H52" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C53" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D53">
         <v>99</v>
       </c>
       <c r="E53" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F53" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G53" t="s">
+        <v>10</v>
+      </c>
+      <c r="H53" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C54" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D54">
         <v>127</v>
       </c>
       <c r="E54" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F54" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G54" t="s">
+        <v>10</v>
+      </c>
+      <c r="H54" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C55" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D55">
         <v>122</v>
       </c>
       <c r="E55" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F55" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G55" t="s">
+        <v>10</v>
+      </c>
+      <c r="H55" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C56" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D56">
         <v>104</v>
       </c>
       <c r="E56" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F56" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G56" t="s">
+        <v>10</v>
+      </c>
+      <c r="H56" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C57" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D57">
         <v>106</v>
       </c>
       <c r="E57" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F57" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G57" t="s">
+        <v>10</v>
+      </c>
+      <c r="H57" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C58" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D58">
         <v>105</v>
       </c>
       <c r="E58" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F58" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G58" t="s">
+        <v>10</v>
+      </c>
+      <c r="H58" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C59" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D59">
         <v>92</v>
       </c>
       <c r="E59" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F59" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G59" t="s">
+        <v>10</v>
+      </c>
+      <c r="H59" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B60" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C60" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D60">
         <v>88</v>
       </c>
       <c r="E60" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F60" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G60" t="s">
+        <v>10</v>
+      </c>
+      <c r="H60" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B61" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C61" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D61">
         <v>101</v>
       </c>
       <c r="E61" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F61" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G61" t="s">
+        <v>10</v>
+      </c>
+      <c r="H61" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C62" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D62">
         <v>126</v>
       </c>
       <c r="E62" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F62" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G62" t="s">
+        <v>10</v>
+      </c>
+      <c r="H62" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C63" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D63">
         <v>80</v>
       </c>
       <c r="E63" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F63" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G63" t="s">
+        <v>10</v>
+      </c>
+      <c r="H63" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C64" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D64">
         <v>95</v>
       </c>
       <c r="E64" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F64" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G64" t="s">
+        <v>10</v>
+      </c>
+      <c r="H64" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B65" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C65" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D65">
         <v>107</v>
       </c>
       <c r="E65" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F65" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G65" t="s">
+        <v>10</v>
+      </c>
+      <c r="H65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B66" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C66" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D66">
         <v>120</v>
       </c>
       <c r="E66" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F66" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G66" t="s">
+        <v>10</v>
+      </c>
+      <c r="H66" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C67" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D67">
         <v>89</v>
       </c>
       <c r="E67" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F67" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G67" t="s">
+        <v>10</v>
+      </c>
+      <c r="H67" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C68" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D68">
         <v>116</v>
       </c>
       <c r="E68" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F68" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G68" t="s">
+        <v>10</v>
+      </c>
+      <c r="H68" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C69" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D69">
         <v>98</v>
       </c>
       <c r="E69" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F69" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G69" t="s">
+        <v>10</v>
+      </c>
+      <c r="H69" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C70" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D70">
         <v>103</v>
       </c>
       <c r="E70" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F70" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G70" t="s">
+        <v>10</v>
+      </c>
+      <c r="H70" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C71" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D71">
         <v>99</v>
       </c>
       <c r="E71" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F71" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G71" t="s">
+        <v>10</v>
+      </c>
+      <c r="H71" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C72" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D72">
         <v>86</v>
       </c>
       <c r="E72" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F72" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="G72" t="s">
+        <v>10</v>
+      </c>
+      <c r="H72" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C73" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D73">
         <v>101</v>
       </c>
       <c r="E73" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F73" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="G73" t="s">
+        <v>10</v>
+      </c>
+      <c r="H73" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="74" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B74" t="s">
+        <v>153</v>
+      </c>
+      <c r="C74" t="s">
+        <v>154</v>
+      </c>
+      <c r="D74">
+        <v>89</v>
+      </c>
+      <c r="E74" t="s">
+        <v>10</v>
+      </c>
+      <c r="F74" t="s">
+        <v>10</v>
+      </c>
+      <c r="G74" t="s">
+        <v>10</v>
+      </c>
+      <c r="H74" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="75" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B75" t="s">
+        <v>155</v>
+      </c>
+      <c r="C75" t="s">
+        <v>156</v>
+      </c>
+      <c r="D75">
+        <v>81</v>
+      </c>
+      <c r="E75" t="s">
+        <v>10</v>
+      </c>
+      <c r="F75" t="s">
+        <v>10</v>
+      </c>
+      <c r="G75" t="s">
+        <v>10</v>
+      </c>
+      <c r="H75" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B76" t="s">
+        <v>157</v>
+      </c>
+      <c r="C76" t="s">
+        <v>158</v>
+      </c>
+      <c r="D76">
+        <v>74</v>
+      </c>
+      <c r="E76" t="s">
+        <v>10</v>
+      </c>
+      <c r="F76" t="s">
+        <v>10</v>
+      </c>
+      <c r="G76" t="s">
+        <v>10</v>
+      </c>
+      <c r="H76" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="77" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B77" t="s">
+        <v>159</v>
+      </c>
+      <c r="C77" t="s">
+        <v>160</v>
+      </c>
+      <c r="D77">
+        <v>102</v>
+      </c>
+      <c r="E77" t="s">
+        <v>10</v>
+      </c>
+      <c r="F77" t="s">
+        <v>10</v>
+      </c>
+      <c r="G77" t="s">
+        <v>10</v>
+      </c>
+      <c r="H77" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="78" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B78" t="s">
+        <v>161</v>
+      </c>
+      <c r="C78" t="s">
+        <v>162</v>
+      </c>
+      <c r="D78">
+        <v>99</v>
+      </c>
+      <c r="E78" t="s">
+        <v>10</v>
+      </c>
+      <c r="F78" t="s">
+        <v>10</v>
+      </c>
+      <c r="G78" t="s">
+        <v>10</v>
+      </c>
+      <c r="H78" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B79" t="s">
+        <v>163</v>
+      </c>
+      <c r="C79" t="s">
+        <v>164</v>
+      </c>
+      <c r="D79">
+        <v>83</v>
+      </c>
+      <c r="E79" t="s">
+        <v>10</v>
+      </c>
+      <c r="F79" t="s">
+        <v>10</v>
+      </c>
+      <c r="G79" t="s">
+        <v>10</v>
+      </c>
+      <c r="H79" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="80" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B80" t="s">
+        <v>165</v>
+      </c>
+      <c r="C80" t="s">
+        <v>166</v>
+      </c>
+      <c r="D80">
+        <v>104</v>
+      </c>
+      <c r="E80" t="s">
+        <v>10</v>
+      </c>
+      <c r="F80" t="s">
+        <v>10</v>
+      </c>
+      <c r="G80" t="s">
+        <v>10</v>
+      </c>
+      <c r="H80" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B81" t="s">
+        <v>167</v>
+      </c>
+      <c r="C81" t="s">
+        <v>168</v>
+      </c>
+      <c r="D81">
+        <v>80</v>
+      </c>
+      <c r="E81" t="s">
+        <v>10</v>
+      </c>
+      <c r="F81" t="s">
+        <v>10</v>
+      </c>
+      <c r="G81" t="s">
+        <v>10</v>
+      </c>
+      <c r="H81" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B82" t="s">
+        <v>169</v>
+      </c>
+      <c r="C82" t="s">
+        <v>170</v>
+      </c>
+      <c r="D82">
+        <v>79</v>
+      </c>
+      <c r="E82" t="s">
+        <v>10</v>
+      </c>
+      <c r="F82" t="s">
+        <v>10</v>
+      </c>
+      <c r="G82" t="s">
+        <v>10</v>
+      </c>
+      <c r="H82" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B83" t="s">
+        <v>171</v>
+      </c>
+      <c r="C83" t="s">
+        <v>172</v>
+      </c>
+      <c r="D83">
+        <v>102</v>
+      </c>
+      <c r="E83" t="s">
+        <v>10</v>
+      </c>
+      <c r="F83" t="s">
+        <v>10</v>
+      </c>
+      <c r="G83" t="s">
+        <v>10</v>
+      </c>
+      <c r="H83" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B84" t="s">
+        <v>173</v>
+      </c>
+      <c r="C84" t="s">
+        <v>174</v>
+      </c>
+      <c r="D84">
+        <v>93</v>
+      </c>
+      <c r="E84" t="s">
+        <v>10</v>
+      </c>
+      <c r="F84" t="s">
+        <v>10</v>
+      </c>
+      <c r="G84" t="s">
+        <v>10</v>
+      </c>
+      <c r="H84" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B85" t="s">
+        <v>175</v>
+      </c>
+      <c r="C85" t="s">
+        <v>176</v>
+      </c>
+      <c r="D85">
+        <v>81</v>
+      </c>
+      <c r="E85" t="s">
+        <v>10</v>
+      </c>
+      <c r="F85" t="s">
+        <v>10</v>
+      </c>
+      <c r="G85" t="s">
+        <v>10</v>
+      </c>
+      <c r="H85" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A98" s="1"/>
+      <c r="A98" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A123">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
+        <v>223</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFEB26E8-D75F-4248-829F-C634CCC56C68}">
-  <dimension ref="A1:G46"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2">
-        <v>7127</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
-        <v>0.97390046296296295</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="2">
-        <v>2020</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>